<commit_message>
mark WebCatalogue consolidation complete
</commit_message>
<xml_diff>
--- a/docs/checklist - roadmap organizado.xlsx
+++ b/docs/checklist - roadmap organizado.xlsx
@@ -832,9 +832,9 @@
           <t xml:space="preserve">Consolidar alterações locais em commits por tema</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr" s="4">
-        <is>
-          <t xml:space="preserve">Em curso</t>
+      <c r="E3" t="inlineStr" s="3">
+        <is>
+          <t xml:space="preserve">Feito</t>
         </is>
       </c>
       <c r="F3" t="inlineStr" s="2">
@@ -849,7 +849,7 @@
       </c>
       <c r="H3" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Inventariar alterações; excluir __pycache__ e .pyc; separar commits por tema</t>
+          <t xml:space="preserve">Concluído em 2026-07-25: 15275fd0 higiene; 97f0910e frontoffice/benchmark; ce6cf863 documentação/roadmap</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
preserve PHPUnit environment during bootstrap
</commit_message>
<xml_diff>
--- a/docs/checklist - roadmap organizado.xlsx
+++ b/docs/checklist - roadmap organizado.xlsx
@@ -874,9 +874,9 @@
           <t xml:space="preserve">Corrigir HTTP 419/CSRF na suite WebCatalogue</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Pendente</t>
+      <c r="E4" t="inlineStr" s="3">
+        <is>
+          <t xml:space="preserve">Feito</t>
         </is>
       </c>
       <c r="F4" t="inlineStr" s="2">
@@ -891,7 +891,7 @@
       </c>
       <c r="H4" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Usar base de dados isolada</t>
+          <t xml:space="preserve">Concluído em 2026-07-25: 4 testes, 20 asserções; bootstrap preserva APP_ENV=testing em CLI</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
add WebCatalogue public journey regression test
</commit_message>
<xml_diff>
--- a/docs/checklist - roadmap organizado.xlsx
+++ b/docs/checklist - roadmap organizado.xlsx
@@ -916,9 +916,9 @@
           <t xml:space="preserve">Validar percurso E2E atual em desktop e telemóvel</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Pendente</t>
+      <c r="E5" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Em curso</t>
         </is>
       </c>
       <c r="F5" t="inlineStr" s="2">
@@ -933,7 +933,7 @@
       </c>
       <c r="H5" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Guardar evidência</t>
+          <t xml:space="preserve">HTTP desktop/mobile e testes automáticos concluídos: 5 testes/44 asserções; falta validação visual, JS e câmara em dispositivos reais</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
complete WebCatalogue end-to-end validation
</commit_message>
<xml_diff>
--- a/docs/checklist - roadmap organizado.xlsx
+++ b/docs/checklist - roadmap organizado.xlsx
@@ -916,9 +916,9 @@
           <t xml:space="preserve">Validar percurso E2E atual em desktop e telemóvel</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr" s="4">
-        <is>
-          <t xml:space="preserve">Em curso</t>
+      <c r="E5" t="inlineStr" s="3">
+        <is>
+          <t xml:space="preserve">Feito</t>
         </is>
       </c>
       <c r="F5" t="inlineStr" s="2">
@@ -933,7 +933,7 @@
       </c>
       <c r="H5" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">HTTP desktop/mobile e testes automáticos concluídos: 5 testes/44 asserções; falta validação visual, JS e câmara em dispositivos reais</t>
+          <t xml:space="preserve">Concluído em 2026-07-25: 5 testes/44 asserções e validação manual desktop/mobile confirmada sem erros bloqueadores</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
inventory WebCatalogue backoffice dependencies
</commit_message>
<xml_diff>
--- a/docs/checklist - roadmap organizado.xlsx
+++ b/docs/checklist - roadmap organizado.xlsx
@@ -958,9 +958,9 @@
           <t xml:space="preserve">Inventariar dependências no BO agregador</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Pendente</t>
+      <c r="E6" t="inlineStr" s="3">
+        <is>
+          <t xml:space="preserve">Feito</t>
         </is>
       </c>
       <c r="F6" t="inlineStr" s="2">
@@ -975,7 +975,7 @@
       </c>
       <c r="H6" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">App, SiteManager, auth, layouts, notifications e tools</t>
+          <t xml:space="preserve">Concluído em 2026-07-25: 27 controllers, 45 views BO e dependências auth, permissions, notifications, module loader, storage, queues, AI e MTG classificadas</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
propose WebCatalogue multi-tenant model
</commit_message>
<xml_diff>
--- a/docs/checklist - roadmap organizado.xlsx
+++ b/docs/checklist - roadmap organizado.xlsx
@@ -1000,9 +1000,9 @@
           <t xml:space="preserve">Definir multi-tenancy por organização e store</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Pendente</t>
+      <c r="E7" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Em curso</t>
         </is>
       </c>
       <c r="F7" t="inlineStr" s="2">
@@ -1017,7 +1017,7 @@
       </c>
       <c r="H7" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Cobrir utilizadores com várias stores</t>
+          <t xml:space="preserve">Proposta criada em docs/webcatalogue_multitenancy_model.md; aguarda aprovação das decisões de tenancy</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
approve WebCatalogue multi-tenant model
</commit_message>
<xml_diff>
--- a/docs/checklist - roadmap organizado.xlsx
+++ b/docs/checklist - roadmap organizado.xlsx
@@ -1000,9 +1000,9 @@
           <t xml:space="preserve">Definir multi-tenancy por organização e store</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr" s="4">
-        <is>
-          <t xml:space="preserve">Em curso</t>
+      <c r="E7" t="inlineStr" s="3">
+        <is>
+          <t xml:space="preserve">Feito</t>
         </is>
       </c>
       <c r="F7" t="inlineStr" s="2">
@@ -1017,7 +1017,7 @@
       </c>
       <c r="H7" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Proposta criada em docs/webcatalogue_multitenancy_model.md; aguarda aprovação das decisões de tenancy</t>
+          <t xml:space="preserve">Aprovado em 2026-07-25: organização como tenant, store operacional, isolamento por linha e TenantContext obrigatório</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
propose WebCatalogue access control model
</commit_message>
<xml_diff>
--- a/docs/checklist - roadmap organizado.xlsx
+++ b/docs/checklist - roadmap organizado.xlsx
@@ -1042,9 +1042,9 @@
           <t xml:space="preserve">Definir autenticação, SSO, papéis e permissões</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Pendente</t>
+      <c r="E8" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Em curso</t>
         </is>
       </c>
       <c r="F8" t="inlineStr" s="2">
@@ -1059,7 +1059,7 @@
       </c>
       <c r="H8" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Incluir integradores e operadores</t>
+          <t xml:space="preserve">Proposta criada em docs/webcatalogue_auth_roles_permissions.md; aguarda aprovação de roles, policies, MFA, sessões e API scopes</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
approve WebCatalogue access control model
</commit_message>
<xml_diff>
--- a/docs/checklist - roadmap organizado.xlsx
+++ b/docs/checklist - roadmap organizado.xlsx
@@ -1042,9 +1042,9 @@
           <t xml:space="preserve">Definir autenticação, SSO, papéis e permissões</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr" s="4">
-        <is>
-          <t xml:space="preserve">Em curso</t>
+      <c r="E8" t="inlineStr" s="3">
+        <is>
+          <t xml:space="preserve">Feito</t>
         </is>
       </c>
       <c r="F8" t="inlineStr" s="2">
@@ -1059,7 +1059,7 @@
       </c>
       <c r="H8" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Proposta criada em docs/webcatalogue_auth_roles_permissions.md; aguarda aprovação de roles, policies, MFA, sessões e API scopes</t>
+          <t xml:space="preserve">Aprovado em 2026-07-25: auth local, convites, MFA control, roles organização/store, policies, sessões isoladas e API scopes</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
propose phased WebCatalogue backoffice extraction
</commit_message>
<xml_diff>
--- a/docs/checklist - roadmap organizado.xlsx
+++ b/docs/checklist - roadmap organizado.xlsx
@@ -1084,9 +1084,9 @@
           <t xml:space="preserve">Definir plano faseado de extração do BO</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Pendente</t>
+      <c r="E9" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Em curso</t>
         </is>
       </c>
       <c r="F9" t="inlineStr" s="2">
@@ -1101,7 +1101,7 @@
       </c>
       <c r="H9" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Evitar interrupção do sistema atual</t>
+          <t xml:space="preserve">Proposta criada em docs/webcatalogue_backoffice_extraction_plan.md; aguarda aprovação da migração incremental e estratégia de rollback</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
approve fork and prune extraction plan
</commit_message>
<xml_diff>
--- a/docs/checklist - roadmap organizado.xlsx
+++ b/docs/checklist - roadmap organizado.xlsx
@@ -1084,9 +1084,9 @@
           <t xml:space="preserve">Definir plano faseado de extração do BO</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr" s="4">
-        <is>
-          <t xml:space="preserve">Em curso</t>
+      <c r="E9" t="inlineStr" s="3">
+        <is>
+          <t xml:space="preserve">Feito</t>
         </is>
       </c>
       <c r="F9" t="inlineStr" s="2">
@@ -1101,19 +1101,19 @@
       </c>
       <c r="H9" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Plano revisto: fork do BO para repo/servidor próprios, poda do novo BO, migração seletiva e remoção WebCatalogue no BO original após cutover</t>
+          <t xml:space="preserve">Aprovado em 2026-07-25: fork para repo/servidor próprios, poda controlada, migração seletiva e remoção no BO original após cutover</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">S3.1</t>
+          <t xml:space="preserve">S2.5</t>
         </is>
       </c>
       <c r="B10" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">3. Domínio e infraestrutura</t>
+          <t xml:space="preserve">2. Arquitetura autónoma</t>
         </is>
       </c>
       <c r="C10" t="inlineStr" s="2">
@@ -1123,39 +1123,39 @@
       </c>
       <c r="D10" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Definir domínio/subdomínios e ambientes</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr" s="3">
-        <is>
-          <t xml:space="preserve">Feito</t>
+          <t xml:space="preserve">Criar baseline e tag para a separação</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Em curso</t>
         </is>
       </c>
       <c r="F10" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">S2.4</t>
         </is>
       </c>
       <c r="G10" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">URLs finais aprovados</t>
+          <t xml:space="preserve">Suite verde, working tree limpo e tag criada</t>
         </is>
       </c>
       <c r="H10" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Landing: raiz; clientes: studio; admin: control; documentação/API: api; lojas: {store}; www redireciona para raiz</t>
+          <t xml:space="preserve">Preparar baseline webcatalogue-extraction-baseline-2026-07-25</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">S3.2</t>
+          <t xml:space="preserve">S2.6</t>
         </is>
       </c>
       <c r="B11" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">3. Domínio e infraestrutura</t>
+          <t xml:space="preserve">2. Arquitetura autónoma</t>
         </is>
       </c>
       <c r="C11" t="inlineStr" s="2">
@@ -1165,7 +1165,7 @@
       </c>
       <c r="D11" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Configurar DNS principal, subdomínios reservados e wildcard</t>
+          <t xml:space="preserve">Criar novo repositório e ambiente WebCatalogue</t>
         </is>
       </c>
       <c r="E11" t="inlineStr" s="5">
@@ -1175,29 +1175,29 @@
       </c>
       <c r="F11" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">S3.1</t>
+          <t xml:space="preserve">S2.5</t>
         </is>
       </c>
       <c r="G11" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Raiz, studio, control, api e qualquer slug resolvem para o ambiente correto</t>
+          <t xml:space="preserve">Clone funcional em staging com infra própria</t>
         </is>
       </c>
       <c r="H11" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Criar *.ar-webcatalogue.com; reservar www, studio, control, api, status e staging</t>
+          <t xml:space="preserve">Requer destino Git, servidor, DB, storage, secrets e deploy próprios</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">S3.2a</t>
+          <t xml:space="preserve">S2.7</t>
         </is>
       </c>
       <c r="B12" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">3. Domínio e infraestrutura</t>
+          <t xml:space="preserve">2. Arquitetura autónoma</t>
         </is>
       </c>
       <c r="C12" t="inlineStr" s="2">
@@ -1207,7 +1207,7 @@
       </c>
       <c r="D12" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Configurar TLS para raiz e wildcard</t>
+          <t xml:space="preserve">Inventariar e aprovar a poda do novo BO</t>
         </is>
       </c>
       <c r="E12" t="inlineStr" s="5">
@@ -1217,24 +1217,24 @@
       </c>
       <c r="F12" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">S3.2</t>
+          <t xml:space="preserve">S2.6</t>
         </is>
       </c>
       <c r="G12" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">HTTPS válido na raiz, subdomínios técnicos e store de teste</t>
+          <t xml:space="preserve">Todos os módulos classificados</t>
         </is>
       </c>
       <c r="H12" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Cobrir ar-webcatalogue.com e *.ar-webcatalogue.com; renovação automática</t>
+          <t xml:space="preserve">Manter, substituir, remover ou avaliar; mapear dependências transitivas</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">S3.2b</t>
+          <t xml:space="preserve">S3.1</t>
         </is>
       </c>
       <c r="B13" t="inlineStr" s="2">
@@ -1249,34 +1249,34 @@
       </c>
       <c r="D13" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Configurar virtual host/reverse proxy wildcard</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Pendente</t>
+          <t xml:space="preserve">Definir domínio/subdomínios e ambientes</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr" s="3">
+        <is>
+          <t xml:space="preserve">Feito</t>
         </is>
       </c>
       <c r="F13" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">S3.2, S3.2a</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="G13" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Hosts técnicos e stores chegam à aplicação correta</t>
+          <t xml:space="preserve">URLs finais aprovados</t>
         </is>
       </c>
       <c r="H13" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Aceitar apenas primeiro nível; rejeitar hosts inválidos</t>
+          <t xml:space="preserve">Landing: raiz; clientes: studio; admin: control; documentação/API: api; lojas: {store}; www redireciona para raiz</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">S3.2c</t>
+          <t xml:space="preserve">S3.2</t>
         </is>
       </c>
       <c r="B14" t="inlineStr" s="2">
@@ -1291,7 +1291,7 @@
       </c>
       <c r="D14" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Implementar resolução automática da store pelo hostname</t>
+          <t xml:space="preserve">Configurar DNS principal, subdomínios reservados e wildcard</t>
         </is>
       </c>
       <c r="E14" t="inlineStr" s="5">
@@ -1301,24 +1301,24 @@
       </c>
       <c r="F14" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">S2.2, S3.2b</t>
+          <t xml:space="preserve">S3.1</t>
         </is>
       </c>
       <c r="G14" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Hostname resolve exatamente uma store ativa e isola os dados</t>
+          <t xml:space="preserve">Raiz, studio, control, api e qualquer slug resolvem para o ambiente correto</t>
         </is>
       </c>
       <c r="H14" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não confiar em store_id enviado pelo cliente</t>
+          <t xml:space="preserve">Criar *.ar-webcatalogue.com; reservar www, studio, control, api, status e staging</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">S3.2d</t>
+          <t xml:space="preserve">S3.2a</t>
         </is>
       </c>
       <c r="B15" t="inlineStr" s="2">
@@ -1333,7 +1333,7 @@
       </c>
       <c r="D15" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Implementar validação, reserva e ciclo de vida do slug</t>
+          <t xml:space="preserve">Configurar TLS para raiz e wildcard</t>
         </is>
       </c>
       <c r="E15" t="inlineStr" s="5">
@@ -1343,24 +1343,24 @@
       </c>
       <c r="F15" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">S3.1, S3.2c</t>
+          <t xml:space="preserve">S3.2</t>
         </is>
       </c>
       <c r="G15" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Slug único cria URL automaticamente; rename/delete são seguros</t>
+          <t xml:space="preserve">HTTPS válido na raiz, subdomínios técnicos e store de teste</t>
         </is>
       </c>
       <c r="H15" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Bloquear nomes técnicos; prevenir subdomain takeover; redirecionar rename quando aplicável</t>
+          <t xml:space="preserve">Cobrir ar-webcatalogue.com e *.ar-webcatalogue.com; renovação automática</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">S3.3</t>
+          <t xml:space="preserve">S3.2b</t>
         </is>
       </c>
       <c r="B16" t="inlineStr" s="2">
@@ -1375,7 +1375,7 @@
       </c>
       <c r="D16" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Configurar sessões, cookies, CORS e CSRF por hostname</t>
+          <t xml:space="preserve">Configurar virtual host/reverse proxy wildcard</t>
         </is>
       </c>
       <c r="E16" t="inlineStr" s="5">
@@ -1385,24 +1385,24 @@
       </c>
       <c r="F16" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">S3.2b</t>
+          <t xml:space="preserve">S3.2, S3.2a</t>
         </is>
       </c>
       <c r="G16" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Login, API e catálogos funcionam apenas entre origens autorizadas</t>
+          <t xml:space="preserve">Hosts técnicos e stores chegam à aplicação correta</t>
         </is>
       </c>
       <c r="H16" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Cookies isolados em studio e control; stores públicas sem sessão partilhada</t>
+          <t xml:space="preserve">Aceitar apenas primeiro nível; rejeitar hosts inválidos</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">S3.4</t>
+          <t xml:space="preserve">S3.2c</t>
         </is>
       </c>
       <c r="B17" t="inlineStr" s="2">
@@ -1412,12 +1412,12 @@
       </c>
       <c r="C17" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Média</t>
+          <t xml:space="preserve">Alta</t>
         </is>
       </c>
       <c r="D17" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Preparar deploy, backup, restore e observabilidade</t>
+          <t xml:space="preserve">Implementar resolução automática da store pelo hostname</t>
         </is>
       </c>
       <c r="E17" t="inlineStr" s="5">
@@ -1427,29 +1427,29 @@
       </c>
       <c r="F17" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">S3.2b</t>
+          <t xml:space="preserve">S2.2, S3.2b</t>
         </is>
       </c>
       <c r="G17" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Deploy e restore testados</t>
+          <t xml:space="preserve">Hostname resolve exatamente uma store ativa e isola os dados</t>
         </is>
       </c>
       <c r="H17" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Logs por hostname/store sem tokens ou dados sensíveis</t>
+          <t xml:space="preserve">Não confiar em store_id enviado pelo cliente</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">S4.1</t>
+          <t xml:space="preserve">S3.2d</t>
         </is>
       </c>
       <c r="B18" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">4. Backoffice autónomo</t>
+          <t xml:space="preserve">3. Domínio e infraestrutura</t>
         </is>
       </c>
       <c r="C18" t="inlineStr" s="2">
@@ -1459,7 +1459,7 @@
       </c>
       <c r="D18" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Criar shell visual e navegação próprias</t>
+          <t xml:space="preserve">Implementar validação, reserva e ciclo de vida do slug</t>
         </is>
       </c>
       <c r="E18" t="inlineStr" s="5">
@@ -1469,29 +1469,29 @@
       </c>
       <c r="F18" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">S2.4, S3.2b</t>
+          <t xml:space="preserve">S3.1, S3.2c</t>
         </is>
       </c>
       <c r="G18" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">BO abre sem layout agregador</t>
+          <t xml:space="preserve">Slug único cria URL automaticamente; rename/delete são seguros</t>
         </is>
       </c>
       <c r="H18" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">studio para clientes; control para administração interna</t>
+          <t xml:space="preserve">Bloquear nomes técnicos; prevenir subdomain takeover; redirecionar rename quando aplicável</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">S4.2</t>
+          <t xml:space="preserve">S3.3</t>
         </is>
       </c>
       <c r="B19" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">4. Backoffice autónomo</t>
+          <t xml:space="preserve">3. Domínio e infraestrutura</t>
         </is>
       </c>
       <c r="C19" t="inlineStr" s="2">
@@ -1501,7 +1501,7 @@
       </c>
       <c r="D19" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Migrar autenticação, autorização e gestão de conta</t>
+          <t xml:space="preserve">Configurar sessões, cookies, CORS e CSRF por hostname</t>
         </is>
       </c>
       <c r="E19" t="inlineStr" s="5">
@@ -1511,39 +1511,39 @@
       </c>
       <c r="F19" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">S2.3, S4.1</t>
+          <t xml:space="preserve">S3.2b</t>
         </is>
       </c>
       <c r="G19" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Acessos por papel validados</t>
+          <t xml:space="preserve">Login, API e catálogos funcionam apenas entre origens autorizadas</t>
         </is>
       </c>
       <c r="H19" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Incluir recuperação de password</t>
+          <t xml:space="preserve">Cookies isolados em studio e control; stores públicas sem sessão partilhada</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">S4.3</t>
+          <t xml:space="preserve">S3.4</t>
         </is>
       </c>
       <c r="B20" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">4. Backoffice autónomo</t>
+          <t xml:space="preserve">3. Domínio e infraestrutura</t>
         </is>
       </c>
       <c r="C20" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Alta</t>
+          <t xml:space="preserve">Média</t>
         </is>
       </c>
       <c r="D20" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Migrar todas as áreas e rotas administrativas</t>
+          <t xml:space="preserve">Preparar deploy, backup, restore e observabilidade</t>
         </is>
       </c>
       <c r="E20" t="inlineStr" s="5">
@@ -1553,24 +1553,24 @@
       </c>
       <c r="F20" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">S4.1, S4.2</t>
+          <t xml:space="preserve">S3.2b</t>
         </is>
       </c>
       <c r="G20" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Paridade funcional validada</t>
+          <t xml:space="preserve">Deploy e restore testados</t>
         </is>
       </c>
       <c r="H20" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Remover links para BO agregador</t>
+          <t xml:space="preserve">Logs por hostname/store sem tokens ou dados sensíveis</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">S4.4</t>
+          <t xml:space="preserve">S4.1</t>
         </is>
       </c>
       <c r="B21" t="inlineStr" s="2">
@@ -1580,12 +1580,12 @@
       </c>
       <c r="C21" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Média</t>
+          <t xml:space="preserve">Alta</t>
         </is>
       </c>
       <c r="D21" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Criar dashboard operacional próprio</t>
+          <t xml:space="preserve">Criar shell visual e navegação próprias</t>
         </is>
       </c>
       <c r="E21" t="inlineStr" s="5">
@@ -1595,29 +1595,29 @@
       </c>
       <c r="F21" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">S4.3</t>
+          <t xml:space="preserve">S2.4, S3.2b</t>
         </is>
       </c>
       <c r="G21" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Estado de stores, sync e reconhecimento visível</t>
+          <t xml:space="preserve">BO abre sem layout agregador</t>
         </is>
       </c>
       <c r="H21" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Ações principais acessíveis</t>
+          <t xml:space="preserve">studio para clientes; control para administração interna</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">S5.1</t>
+          <t xml:space="preserve">S4.2</t>
         </is>
       </c>
       <c r="B22" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">5. Instalação de lojas</t>
+          <t xml:space="preserve">4. Backoffice autónomo</t>
         </is>
       </c>
       <c r="C22" t="inlineStr" s="2">
@@ -1627,7 +1627,7 @@
       </c>
       <c r="D22" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Criar organização, store e equipa</t>
+          <t xml:space="preserve">Migrar autenticação, autorização e gestão de conta</t>
         </is>
       </c>
       <c r="E22" t="inlineStr" s="5">
@@ -1637,29 +1637,29 @@
       </c>
       <c r="F22" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">S4.2</t>
+          <t xml:space="preserve">S2.3, S4.1</t>
         </is>
       </c>
       <c r="G22" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Store isolada criada</t>
+          <t xml:space="preserve">Acessos por papel validados</t>
         </is>
       </c>
       <c r="H22" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Convites e papéis</t>
+          <t xml:space="preserve">Incluir recuperação de password</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">S5.2</t>
+          <t xml:space="preserve">S4.3</t>
         </is>
       </c>
       <c r="B23" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">5. Instalação de lojas</t>
+          <t xml:space="preserve">4. Backoffice autónomo</t>
         </is>
       </c>
       <c r="C23" t="inlineStr" s="2">
@@ -1669,7 +1669,7 @@
       </c>
       <c r="D23" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Criar wizard de onboarding da store</t>
+          <t xml:space="preserve">Migrar todas as áreas e rotas administrativas</t>
         </is>
       </c>
       <c r="E23" t="inlineStr" s="5">
@@ -1679,39 +1679,39 @@
       </c>
       <c r="F23" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">S5.1</t>
+          <t xml:space="preserve">S4.1, S4.2</t>
         </is>
       </c>
       <c r="G23" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Wizard concluído sem ajuda</t>
+          <t xml:space="preserve">Paridade funcional validada</t>
         </is>
       </c>
       <c r="H23" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Guardar progresso</t>
+          <t xml:space="preserve">Remover links para BO agregador</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">S5.3</t>
+          <t xml:space="preserve">S4.4</t>
         </is>
       </c>
       <c r="B24" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">5. Instalação de lojas</t>
+          <t xml:space="preserve">4. Backoffice autónomo</t>
         </is>
       </c>
       <c r="C24" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Alta</t>
+          <t xml:space="preserve">Média</t>
         </is>
       </c>
       <c r="D24" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Configurar branding, idioma, moeda, impostos e domínio</t>
+          <t xml:space="preserve">Criar dashboard operacional próprio</t>
         </is>
       </c>
       <c r="E24" t="inlineStr" s="5">
@@ -1721,24 +1721,24 @@
       </c>
       <c r="F24" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">S5.2</t>
+          <t xml:space="preserve">S4.3</t>
         </is>
       </c>
       <c r="G24" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Preview reflete configuração</t>
+          <t xml:space="preserve">Estado de stores, sync e reconhecimento visível</t>
         </is>
       </c>
       <c r="H24" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Valores por defeito seguros</t>
+          <t xml:space="preserve">Ações principais acessíveis</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">S5.4</t>
+          <t xml:space="preserve">S5.1</t>
         </is>
       </c>
       <c r="B25" t="inlineStr" s="2">
@@ -1753,7 +1753,7 @@
       </c>
       <c r="D25" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Configurar origem de produtos e primeiro catálogo</t>
+          <t xml:space="preserve">Criar organização, store e equipa</t>
         </is>
       </c>
       <c r="E25" t="inlineStr" s="5">
@@ -1763,24 +1763,24 @@
       </c>
       <c r="F25" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">S5.2</t>
+          <t xml:space="preserve">S4.2</t>
         </is>
       </c>
       <c r="G25" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Produtos importados e catálogo criado</t>
+          <t xml:space="preserve">Store isolada criada</t>
         </is>
       </c>
       <c r="H25" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Manual, conector ou API</t>
+          <t xml:space="preserve">Convites e papéis</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">S5.5</t>
+          <t xml:space="preserve">S5.2</t>
         </is>
       </c>
       <c r="B26" t="inlineStr" s="2">
@@ -1795,7 +1795,7 @@
       </c>
       <c r="D26" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Criar checklist de ativação e publicação</t>
+          <t xml:space="preserve">Criar wizard de onboarding da store</t>
         </is>
       </c>
       <c r="E26" t="inlineStr" s="5">
@@ -1805,29 +1805,29 @@
       </c>
       <c r="F26" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">S5.3, S5.4</t>
+          <t xml:space="preserve">S5.1</t>
         </is>
       </c>
       <c r="G26" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Store publicada com validações completas</t>
+          <t xml:space="preserve">Wizard concluído sem ajuda</t>
         </is>
       </c>
       <c r="H26" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Permitir regressar a passos incompletos</t>
+          <t xml:space="preserve">Guardar progresso</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">S6.1</t>
+          <t xml:space="preserve">S5.3</t>
         </is>
       </c>
       <c r="B27" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">6. Frontoffice institucional</t>
+          <t xml:space="preserve">5. Instalação de lojas</t>
         </is>
       </c>
       <c r="C27" t="inlineStr" s="2">
@@ -1837,7 +1837,7 @@
       </c>
       <c r="D27" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Definir conteúdo, público-alvo e proposta de valor</t>
+          <t xml:space="preserve">Configurar branding, idioma, moeda, impostos e domínio</t>
         </is>
       </c>
       <c r="E27" t="inlineStr" s="5">
@@ -1847,29 +1847,29 @@
       </c>
       <c r="F27" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">S0.1</t>
+          <t xml:space="preserve">S5.2</t>
         </is>
       </c>
       <c r="G27" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Copy e estrutura aprovadas</t>
+          <t xml:space="preserve">Preview reflete configuração</t>
         </is>
       </c>
       <c r="H27" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não confundir com catálogo da loja</t>
+          <t xml:space="preserve">Valores por defeito seguros</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">S6.2</t>
+          <t xml:space="preserve">S5.4</t>
         </is>
       </c>
       <c r="B28" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">6. Frontoffice institucional</t>
+          <t xml:space="preserve">5. Instalação de lojas</t>
         </is>
       </c>
       <c r="C28" t="inlineStr" s="2">
@@ -1879,7 +1879,7 @@
       </c>
       <c r="D28" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Criar landing responsiva</t>
+          <t xml:space="preserve">Configurar origem de produtos e primeiro catálogo</t>
         </is>
       </c>
       <c r="E28" t="inlineStr" s="5">
@@ -1889,39 +1889,39 @@
       </c>
       <c r="F28" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">S3.2b, S6.1</t>
+          <t xml:space="preserve">S5.2</t>
         </is>
       </c>
       <c r="G28" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Landing acessível no domínio</t>
+          <t xml:space="preserve">Produtos importados e catálogo criado</t>
         </is>
       </c>
       <c r="H28" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Demo visual, casos de uso e CTA</t>
+          <t xml:space="preserve">Manual, conector ou API</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">S6.3</t>
+          <t xml:space="preserve">S5.5</t>
         </is>
       </c>
       <c r="B29" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">6. Frontoffice institucional</t>
+          <t xml:space="preserve">5. Instalação de lojas</t>
         </is>
       </c>
       <c r="C29" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Média</t>
+          <t xml:space="preserve">Alta</t>
         </is>
       </c>
       <c r="D29" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Criar FAQ, páginas legais, SEO e analytics consentido</t>
+          <t xml:space="preserve">Criar checklist de ativação e publicação</t>
         </is>
       </c>
       <c r="E29" t="inlineStr" s="5">
@@ -1931,24 +1931,24 @@
       </c>
       <c r="F29" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">S6.2</t>
+          <t xml:space="preserve">S5.3, S5.4</t>
         </is>
       </c>
       <c r="G29" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Auditoria legal/SEO concluída</t>
+          <t xml:space="preserve">Store publicada com validações completas</t>
         </is>
       </c>
       <c r="H29" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Privacidade e cookies</t>
+          <t xml:space="preserve">Permitir regressar a passos incompletos</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">S6.4</t>
+          <t xml:space="preserve">S6.1</t>
         </is>
       </c>
       <c r="B30" t="inlineStr" s="2">
@@ -1963,7 +1963,7 @@
       </c>
       <c r="D30" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Ligar CTA a demo, registo, login ou contacto</t>
+          <t xml:space="preserve">Definir conteúdo, público-alvo e proposta de valor</t>
         </is>
       </c>
       <c r="E30" t="inlineStr" s="5">
@@ -1973,29 +1973,29 @@
       </c>
       <c r="F30" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">S5.2, S6.2</t>
+          <t xml:space="preserve">S0.1</t>
         </is>
       </c>
       <c r="G30" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lead/onboarding criado corretamente</t>
+          <t xml:space="preserve">Copy e estrutura aprovadas</t>
         </is>
       </c>
       <c r="H30" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Medir conversão</t>
+          <t xml:space="preserve">Não confundir com catálogo da loja</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">S7.1</t>
+          <t xml:space="preserve">S6.2</t>
         </is>
       </c>
       <c r="B31" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">7. API pública v1</t>
+          <t xml:space="preserve">6. Frontoffice institucional</t>
         </is>
       </c>
       <c r="C31" t="inlineStr" s="2">
@@ -2005,7 +2005,7 @@
       </c>
       <c r="D31" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Definir recursos, contratos e versionamento OpenAPI</t>
+          <t xml:space="preserve">Criar landing responsiva</t>
         </is>
       </c>
       <c r="E31" t="inlineStr" s="5">
@@ -2015,39 +2015,39 @@
       </c>
       <c r="F31" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">S2.2</t>
+          <t xml:space="preserve">S3.2b, S6.1</t>
         </is>
       </c>
       <c r="G31" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Especificação v1 aprovada</t>
+          <t xml:space="preserve">Landing acessível no domínio</t>
         </is>
       </c>
       <c r="H31" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Stores, catálogos, produtos, preço, stock e media</t>
+          <t xml:space="preserve">Demo visual, casos de uso e CTA</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">S7.2</t>
+          <t xml:space="preserve">S6.3</t>
         </is>
       </c>
       <c r="B32" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">7. API pública v1</t>
+          <t xml:space="preserve">6. Frontoffice institucional</t>
         </is>
       </c>
       <c r="C32" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Alta</t>
+          <t xml:space="preserve">Média</t>
         </is>
       </c>
       <c r="D32" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Implementar autenticação, scopes e credenciais por store</t>
+          <t xml:space="preserve">Criar FAQ, páginas legais, SEO e analytics consentido</t>
         </is>
       </c>
       <c r="E32" t="inlineStr" s="5">
@@ -2057,29 +2057,29 @@
       </c>
       <c r="F32" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">S2.3, S7.1</t>
+          <t xml:space="preserve">S6.2</t>
         </is>
       </c>
       <c r="G32" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Isolamento e revogação testados</t>
+          <t xml:space="preserve">Auditoria legal/SEO concluída</t>
         </is>
       </c>
       <c r="H32" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Rotação sem downtime</t>
+          <t xml:space="preserve">Privacidade e cookies</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">S7.3</t>
+          <t xml:space="preserve">S6.4</t>
         </is>
       </c>
       <c r="B33" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">7. API pública v1</t>
+          <t xml:space="preserve">6. Frontoffice institucional</t>
         </is>
       </c>
       <c r="C33" t="inlineStr" s="2">
@@ -2089,7 +2089,7 @@
       </c>
       <c r="D33" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Implementar endpoints de catálogo e publicação</t>
+          <t xml:space="preserve">Ligar CTA a demo, registo, login ou contacto</t>
         </is>
       </c>
       <c r="E33" t="inlineStr" s="5">
@@ -2099,24 +2099,24 @@
       </c>
       <c r="F33" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">S7.1, S7.2</t>
+          <t xml:space="preserve">S5.2, S6.2</t>
         </is>
       </c>
       <c r="G33" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Fluxo custom completo por API</t>
+          <t xml:space="preserve">Lead/onboarding criado corretamente</t>
         </is>
       </c>
       <c r="H33" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Paginação, filtros e erros normalizados</t>
+          <t xml:space="preserve">Medir conversão</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">S7.4</t>
+          <t xml:space="preserve">S7.1</t>
         </is>
       </c>
       <c r="B34" t="inlineStr" s="2">
@@ -2131,7 +2131,7 @@
       </c>
       <c r="D34" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Implementar idempotência, rate limiting e auditoria</t>
+          <t xml:space="preserve">Definir recursos, contratos e versionamento OpenAPI</t>
         </is>
       </c>
       <c r="E34" t="inlineStr" s="5">
@@ -2141,24 +2141,24 @@
       </c>
       <c r="F34" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">S7.2, S7.3</t>
+          <t xml:space="preserve">S2.2</t>
         </is>
       </c>
       <c r="G34" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Retries não duplicam dados</t>
+          <t xml:space="preserve">Especificação v1 aprovada</t>
         </is>
       </c>
       <c r="H34" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Logs sem payload sensível</t>
+          <t xml:space="preserve">Stores, catálogos, produtos, preço, stock e media</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">S7.5</t>
+          <t xml:space="preserve">S7.2</t>
         </is>
       </c>
       <c r="B35" t="inlineStr" s="2">
@@ -2173,7 +2173,7 @@
       </c>
       <c r="D35" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Criar documentação em api.ar-webcatalogue.com, exemplos, sandbox e coleção de testes</t>
+          <t xml:space="preserve">Implementar autenticação, scopes e credenciais por store</t>
         </is>
       </c>
       <c r="E35" t="inlineStr" s="5">
@@ -2183,29 +2183,29 @@
       </c>
       <c r="F35" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">S7.3, S7.4</t>
+          <t xml:space="preserve">S2.3, S7.1</t>
         </is>
       </c>
       <c r="G35" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Integrador externo conclui quickstart</t>
+          <t xml:space="preserve">Isolamento e revogação testados</t>
         </is>
       </c>
       <c r="H35" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Raiz com portal; /openapi.json; endpoints em /v1; sem apoio da equipa</t>
+          <t xml:space="preserve">Rotação sem downtime</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">S8.1</t>
+          <t xml:space="preserve">S7.3</t>
         </is>
       </c>
       <c r="B36" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">8. Sincronização</t>
+          <t xml:space="preserve">7. API pública v1</t>
         </is>
       </c>
       <c r="C36" t="inlineStr" s="2">
@@ -2215,7 +2215,7 @@
       </c>
       <c r="D36" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Implementar webhooks assinados e retries</t>
+          <t xml:space="preserve">Implementar endpoints de catálogo e publicação</t>
         </is>
       </c>
       <c r="E36" t="inlineStr" s="5">
@@ -2225,29 +2225,29 @@
       </c>
       <c r="F36" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">S7.3</t>
+          <t xml:space="preserve">S7.1, S7.2</t>
         </is>
       </c>
       <c r="G36" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Entrega e reentrega validadas</t>
+          <t xml:space="preserve">Fluxo custom completo por API</t>
         </is>
       </c>
       <c r="H36" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Dead-letter e replay</t>
+          <t xml:space="preserve">Paginação, filtros e erros normalizados</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">S8.2</t>
+          <t xml:space="preserve">S7.4</t>
         </is>
       </c>
       <c r="B37" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">8. Sincronização</t>
+          <t xml:space="preserve">7. API pública v1</t>
         </is>
       </c>
       <c r="C37" t="inlineStr" s="2">
@@ -2257,7 +2257,7 @@
       </c>
       <c r="D37" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Definir origem de verdade e resolução de conflitos</t>
+          <t xml:space="preserve">Implementar idempotência, rate limiting e auditoria</t>
         </is>
       </c>
       <c r="E37" t="inlineStr" s="5">
@@ -2267,29 +2267,29 @@
       </c>
       <c r="F37" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">S7.1</t>
+          <t xml:space="preserve">S7.2, S7.3</t>
         </is>
       </c>
       <c r="G37" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Regras por campo aprovadas</t>
+          <t xml:space="preserve">Retries não duplicam dados</t>
         </is>
       </c>
       <c r="H37" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Cobrir eliminações e arquivo</t>
+          <t xml:space="preserve">Logs sem payload sensível</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">S8.3</t>
+          <t xml:space="preserve">S7.5</t>
         </is>
       </c>
       <c r="B38" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">8. Sincronização</t>
+          <t xml:space="preserve">7. API pública v1</t>
         </is>
       </c>
       <c r="C38" t="inlineStr" s="2">
@@ -2299,7 +2299,7 @@
       </c>
       <c r="D38" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Criar dashboard de sincronização e recuperação</t>
+          <t xml:space="preserve">Criar documentação em api.ar-webcatalogue.com, exemplos, sandbox e coleção de testes</t>
         </is>
       </c>
       <c r="E38" t="inlineStr" s="5">
@@ -2309,29 +2309,29 @@
       </c>
       <c r="F38" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">S8.1, S8.2</t>
+          <t xml:space="preserve">S7.3, S7.4</t>
         </is>
       </c>
       <c r="G38" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Operador diagnostica e repete falha</t>
+          <t xml:space="preserve">Integrador externo conclui quickstart</t>
         </is>
       </c>
       <c r="H38" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Último sync, erro e cursor</t>
+          <t xml:space="preserve">Raiz com portal; /openapi.json; endpoints em /v1; sem apoio da equipa</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">S9.1</t>
+          <t xml:space="preserve">S8.1</t>
         </is>
       </c>
       <c r="B39" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">9. Framework conectores</t>
+          <t xml:space="preserve">8. Sincronização</t>
         </is>
       </c>
       <c r="C39" t="inlineStr" s="2">
@@ -2341,7 +2341,7 @@
       </c>
       <c r="D39" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Criar contrato e toolkit comum de conectores</t>
+          <t xml:space="preserve">Implementar webhooks assinados e retries</t>
         </is>
       </c>
       <c r="E39" t="inlineStr" s="5">
@@ -2351,29 +2351,29 @@
       </c>
       <c r="F39" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">S7.5, S8.3</t>
+          <t xml:space="preserve">S7.3</t>
         </is>
       </c>
       <c r="G39" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Conector de referência funcional</t>
+          <t xml:space="preserve">Entrega e reentrega validadas</t>
         </is>
       </c>
       <c r="H39" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Mapeamento e lifecycle comuns</t>
+          <t xml:space="preserve">Dead-letter e replay</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">S9.2</t>
+          <t xml:space="preserve">S8.2</t>
         </is>
       </c>
       <c r="B40" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">9. Framework conectores</t>
+          <t xml:space="preserve">8. Sincronização</t>
         </is>
       </c>
       <c r="C40" t="inlineStr" s="2">
@@ -2383,7 +2383,7 @@
       </c>
       <c r="D40" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Criar suite de conformidade para conectores</t>
+          <t xml:space="preserve">Definir origem de verdade e resolução de conflitos</t>
         </is>
       </c>
       <c r="E40" t="inlineStr" s="5">
@@ -2393,29 +2393,29 @@
       </c>
       <c r="F40" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">S9.1</t>
+          <t xml:space="preserve">S7.1</t>
         </is>
       </c>
       <c r="G40" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Testes comuns automatizados</t>
+          <t xml:space="preserve">Regras por campo aprovadas</t>
         </is>
       </c>
       <c r="H40" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Instalação, sync, webhook, erro e remoção</t>
+          <t xml:space="preserve">Cobrir eliminações e arquivo</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">S10.1</t>
+          <t xml:space="preserve">S8.3</t>
         </is>
       </c>
       <c r="B41" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">10. Conectores</t>
+          <t xml:space="preserve">8. Sincronização</t>
         </is>
       </c>
       <c r="C41" t="inlineStr" s="2">
@@ -2425,7 +2425,7 @@
       </c>
       <c r="D41" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Implementar WooCommerce</t>
+          <t xml:space="preserve">Criar dashboard de sincronização e recuperação</t>
         </is>
       </c>
       <c r="E41" t="inlineStr" s="5">
@@ -2435,29 +2435,29 @@
       </c>
       <c r="F41" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">S9.1, S9.2</t>
+          <t xml:space="preserve">S8.1, S8.2</t>
         </is>
       </c>
       <c r="G41" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sandbox passa suite</t>
+          <t xml:space="preserve">Operador diagnostica e repete falha</t>
         </is>
       </c>
       <c r="H41" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Confirmar prioridade comercial</t>
+          <t xml:space="preserve">Último sync, erro e cursor</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">S10.2</t>
+          <t xml:space="preserve">S9.1</t>
         </is>
       </c>
       <c r="B42" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">10. Conectores</t>
+          <t xml:space="preserve">9. Framework conectores</t>
         </is>
       </c>
       <c r="C42" t="inlineStr" s="2">
@@ -2467,7 +2467,7 @@
       </c>
       <c r="D42" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Implementar Shopify</t>
+          <t xml:space="preserve">Criar contrato e toolkit comum de conectores</t>
         </is>
       </c>
       <c r="E42" t="inlineStr" s="5">
@@ -2477,29 +2477,29 @@
       </c>
       <c r="F42" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">S9.1, S9.2</t>
+          <t xml:space="preserve">S7.5, S8.3</t>
         </is>
       </c>
       <c r="G42" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sandbox passa suite</t>
+          <t xml:space="preserve">Conector de referência funcional</t>
         </is>
       </c>
       <c r="H42" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Confirmar prioridade comercial</t>
+          <t xml:space="preserve">Mapeamento e lifecycle comuns</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">S10.3</t>
+          <t xml:space="preserve">S9.2</t>
         </is>
       </c>
       <c r="B43" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">10. Conectores</t>
+          <t xml:space="preserve">9. Framework conectores</t>
         </is>
       </c>
       <c r="C43" t="inlineStr" s="2">
@@ -2509,7 +2509,7 @@
       </c>
       <c r="D43" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Implementar PrestaShop</t>
+          <t xml:space="preserve">Criar suite de conformidade para conectores</t>
         </is>
       </c>
       <c r="E43" t="inlineStr" s="5">
@@ -2519,24 +2519,24 @@
       </c>
       <c r="F43" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">S9.1, S9.2</t>
+          <t xml:space="preserve">S9.1</t>
         </is>
       </c>
       <c r="G43" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sandbox passa suite</t>
+          <t xml:space="preserve">Testes comuns automatizados</t>
         </is>
       </c>
       <c r="H43" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Confirmar prioridade comercial</t>
+          <t xml:space="preserve">Instalação, sync, webhook, erro e remoção</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">S10.4</t>
+          <t xml:space="preserve">S10.1</t>
         </is>
       </c>
       <c r="B44" t="inlineStr" s="2">
@@ -2546,12 +2546,12 @@
       </c>
       <c r="C44" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Média</t>
+          <t xml:space="preserve">Alta</t>
         </is>
       </c>
       <c r="D44" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Implementar Magento/Adobe Commerce</t>
+          <t xml:space="preserve">Implementar WooCommerce</t>
         </is>
       </c>
       <c r="E44" t="inlineStr" s="5">
@@ -2578,12 +2578,12 @@
     <row r="45">
       <c r="A45" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">S12.1</t>
+          <t xml:space="preserve">S10.2</t>
         </is>
       </c>
       <c r="B45" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">12. Testes utilizador</t>
+          <t xml:space="preserve">10. Conectores</t>
         </is>
       </c>
       <c r="C45" t="inlineStr" s="2">
@@ -2593,7 +2593,7 @@
       </c>
       <c r="D45" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Recrutar perfis e preparar consentimento/dados</t>
+          <t xml:space="preserve">Implementar Shopify</t>
         </is>
       </c>
       <c r="E45" t="inlineStr" s="5">
@@ -2603,29 +2603,29 @@
       </c>
       <c r="F45" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Fases 5–11</t>
+          <t xml:space="preserve">S9.1, S9.2</t>
         </is>
       </c>
       <c r="G45" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Amostra e sessões marcadas</t>
+          <t xml:space="preserve">Sandbox passa suite</t>
         </is>
       </c>
       <c r="H45" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Gestor, operador, integrador e visitante</t>
+          <t xml:space="preserve">Confirmar prioridade comercial</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">S12.2</t>
+          <t xml:space="preserve">S10.3</t>
         </is>
       </c>
       <c r="B46" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">12. Testes utilizador</t>
+          <t xml:space="preserve">10. Conectores</t>
         </is>
       </c>
       <c r="C46" t="inlineStr" s="2">
@@ -2635,7 +2635,7 @@
       </c>
       <c r="D46" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Executar tarefas guiadas sem instrução de interface</t>
+          <t xml:space="preserve">Implementar PrestaShop</t>
         </is>
       </c>
       <c r="E46" t="inlineStr" s="5">
@@ -2645,39 +2645,39 @@
       </c>
       <c r="F46" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">S12.1</t>
+          <t xml:space="preserve">S9.1, S9.2</t>
         </is>
       </c>
       <c r="G46" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Métricas completas por tarefa</t>
+          <t xml:space="preserve">Sandbox passa suite</t>
         </is>
       </c>
       <c r="H46" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Tempo, sucesso, erros, ajuda e confiança</t>
+          <t xml:space="preserve">Confirmar prioridade comercial</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">S12.3</t>
+          <t xml:space="preserve">S10.4</t>
         </is>
       </c>
       <c r="B47" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">12. Testes utilizador</t>
+          <t xml:space="preserve">10. Conectores</t>
         </is>
       </c>
       <c r="C47" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Alta</t>
+          <t xml:space="preserve">Média</t>
         </is>
       </c>
       <c r="D47" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Classificar feedback por severidade e frequência</t>
+          <t xml:space="preserve">Implementar Magento/Adobe Commerce</t>
         </is>
       </c>
       <c r="E47" t="inlineStr" s="5">
@@ -2687,64 +2687,190 @@
       </c>
       <c r="F47" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">S12.2</t>
+          <t xml:space="preserve">S9.1, S9.2</t>
         </is>
       </c>
       <c r="G47" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Backlog baseado em evidência</t>
+          <t xml:space="preserve">Sandbox passa suite</t>
         </is>
       </c>
       <c r="H47" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">S0 a S3</t>
+          <t xml:space="preserve">Confirmar prioridade comercial</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr" s="2">
         <is>
+          <t xml:space="preserve">S12.1</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">12. Testes utilizador</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Alta</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Recrutar perfis e preparar consentimento/dados</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Pendente</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Fases 5–11</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Amostra e sessões marcadas</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Gestor, operador, integrador e visitante</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">S12.2</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">12. Testes utilizador</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Alta</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Executar tarefas guiadas sem instrução de interface</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Pendente</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">S12.1</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Métricas completas por tarefa</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Tempo, sucesso, erros, ajuda e confiança</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">S12.3</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">12. Testes utilizador</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Alta</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Classificar feedback por severidade e frequência</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Pendente</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">S12.2</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Backlog baseado em evidência</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">S0 a S3</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr" s="2">
+        <is>
           <t xml:space="preserve">S12.4</t>
         </is>
       </c>
-      <c r="B48" t="inlineStr" s="2">
+      <c r="B51" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">12. Testes utilizador</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Alta</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr" s="2">
+      <c r="C51" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Alta</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Corrigir problemas críticos e repetir testes</t>
         </is>
       </c>
-      <c r="E48" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Pendente</t>
-        </is>
-      </c>
-      <c r="F48" t="inlineStr" s="2">
+      <c r="E51" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Pendente</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">S12.3</t>
         </is>
       </c>
-      <c r="G48" t="inlineStr" s="2">
+      <c r="G51" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Sem S0 e S1 tratados/aceites</t>
         </is>
       </c>
-      <c r="H48" t="inlineStr" s="2">
+      <c r="H51" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Guardar evidência do reteste</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H48"/>
+  <autoFilter ref="A1:H51"/>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
record WebCatalogue extraction baseline
</commit_message>
<xml_diff>
--- a/docs/checklist - roadmap organizado.xlsx
+++ b/docs/checklist - roadmap organizado.xlsx
@@ -1126,9 +1126,9 @@
           <t xml:space="preserve">Criar baseline e tag para a separação</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr" s="4">
-        <is>
-          <t xml:space="preserve">Em curso</t>
+      <c r="E10" t="inlineStr" s="3">
+        <is>
+          <t xml:space="preserve">Feito</t>
         </is>
       </c>
       <c r="F10" t="inlineStr" s="2">
@@ -1143,7 +1143,7 @@
       </c>
       <c r="H10" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Preparar baseline webcatalogue-extraction-baseline-2026-07-25</t>
+          <t xml:space="preserve">Concluído em 2026-07-25: 7 testes/49 asserções; tag webcatalogue-extraction-baseline-2026-07-25</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
record WebCatalogue repository and server targets
</commit_message>
<xml_diff>
--- a/docs/checklist - roadmap organizado.xlsx
+++ b/docs/checklist - roadmap organizado.xlsx
@@ -1168,9 +1168,9 @@
           <t xml:space="preserve">Criar novo repositório e ambiente WebCatalogue</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Pendente</t>
+      <c r="E11" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Em curso</t>
         </is>
       </c>
       <c r="F11" t="inlineStr" s="2">
@@ -1185,7 +1185,7 @@
       </c>
       <c r="H11" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Requer destino Git, servidor, DB, storage, secrets e deploy próprios</t>
+          <t xml:space="preserve">Destinos definidos: GitHub wlavv/webcatalogue privado e servidor Rise-S; falta criar repo e configurar acesso/deploy</t>
         </is>
       </c>
     </row>

</xml_diff>